<commit_message>
docs(tutorials): COMBO-3 — the starter file ships γ, γsat, c, φ and u blank; the reader types all five per zone (before/after screenshots); starting-circle paragraphs shortened; the checks aside and the false γsat claim removed
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/tutorials/files/xslope_earth_dam_fs_time_start.xlsx
+++ b/docs/tutorials/files/xslope_earth_dam_fs_time_start.xlsx
@@ -6794,9 +6794,7 @@
         </is>
       </c>
       <c r="C11" s="3"/>
-      <c r="D11" s="3">
-        <v>21.0</v>
-      </c>
+      <c r="D11" s="3"/>
       <c r="E11" s="3" t="inlineStr">
         <is>
           <t>mc</t>
@@ -6823,11 +6821,7 @@
       <c r="N11" s="3">
         <v>0.0</v>
       </c>
-      <c r="O11" s="3" t="inlineStr">
-        <is>
-          <t>seep</t>
-        </is>
-      </c>
+      <c r="O11" s="3"/>
       <c r="P11" s="3">
         <v>0.0</v>
       </c>
@@ -6918,9 +6912,7 @@
         </is>
       </c>
       <c r="C12" s="3"/>
-      <c r="D12" s="3">
-        <v>20.0</v>
-      </c>
+      <c r="D12" s="3"/>
       <c r="E12" s="3" t="inlineStr">
         <is>
           <t>mc</t>
@@ -6947,11 +6939,7 @@
       <c r="N12" s="3">
         <v>0.0</v>
       </c>
-      <c r="O12" s="3" t="inlineStr">
-        <is>
-          <t>seep</t>
-        </is>
-      </c>
+      <c r="O12" s="3"/>
       <c r="P12" s="3">
         <v>0.0</v>
       </c>

</xml_diff>